<commit_message>
update intershop api test case file
</commit_message>
<xml_diff>
--- a/test-cases/web-app/intershop/intershop-api-test-cases.xlsx
+++ b/test-cases/web-app/intershop/intershop-api-test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\WORK RELATED\PORTFOLIOS\QA\qa artifacts unsorted\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\WORK RELATED\PORTFOLIOS\QA\qa-portfolio\test-cases\web-app\intershop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1CB6F4-D51A-4089-A798-7107D7F87A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC3E955-B378-41C9-8E61-4514D4CD0D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="80">
   <si>
     <t>ID</t>
   </si>
@@ -219,121 +219,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Авторизация:
-Login</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: skillboxadmin
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Password</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: iamfinallytester
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">ДАННЫЕ ИЗМЕНЯЕМЫХ ПОЛЕЙ КАРТОЧКИ ТОВАРА ДО ИЗМЕНЕНИЙ:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">{
-    "name": "Поло для теста",
-    "description": "",
-    "price": "100",
-    "sale_price": "",
-    "images": [
-        {
-            "src": "http://intershop3.skillbox.ru/wp-content/uploads/2026/05/10564528-worried-fat-man-with-pink-shirt-isolated-on-white-background-19.jpg"
-        }
-    ]
-}
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">ДАННЫЕ ИЗМЕНЯЕМЫХ ПОЛЕЙ КАРТОЧКИ ТОВАРА ПОСЛЕ ИЗМЕНЕНИЙ:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>{
-  "name": "Поло мужское для теста",
-  "description": "Тестовое мужское поло для проверки редактирования карточки товара через PUT-запрос.",
-  "price": "85",
-  "sale_price": "85",
-  "images": [
-    {
-      "src": "</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>https://png.pngtree.com/png-clipart/20220815/ourmid/pngtree-mens-white-polo-shirt-for-clothing-model-mockup-and-passport-photo-png-image_6110906.png</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"
-    }
-  ]
-}
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Статус-код ответа: 200 OK.
 В теле ответа возвращается JSON обновлённой карточки товара.
 Поля, переданные в PUT-запросе, обновлены:
@@ -544,40 +429,6 @@
 4. Проверить, что id исходной карточки товара не изменился и имеет такое же значение как в переменной {{productid}}.
 5. Отправить GET-запрос на /api/products/999999.
 6. Проверить, что товар с id = 999999 НЕ был создан или изменён этим PUT-запросом.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-Новое значение поля в PUT запросе
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>{
-  "id": 999999
-}</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Ожидаемый статус-код:
@@ -675,39 +526,6 @@
 2. Проверить статус-код и тело ответа.
 3. Отправить GET-запрос на /api/products/{{productid}}.
 4. Проверить, что поле price не обновилось на значение "hundred".</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Новое значение поля в PUT запросе
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>{
-  "price": hundred
-}</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">
@@ -948,13 +766,6 @@
 4. Проверить, что карточка товара больше не доступна.</t>
   </si>
   <si>
-    <t>Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-ID товара получить из переменной {{productid}}
-Значение переменной `{{productid}}` взять из тестовой карточки товара.</t>
-  </si>
-  <si>
     <t>1. DELETE-запрос успешно удаляет существующую карточку товара.
 В ответе приходит статус-код 200 или 204.
 2. При повторном GET-запросе удалённая карточка товара не возвращается.
@@ -1038,12 +849,6 @@
 3. Проверить тело ответа.</t>
   </si>
   <si>
-    <t>Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-ID товара: `999999999`</t>
-  </si>
-  <si>
     <t xml:space="preserve">Сервер должен вернуть HTTP-статус `404 Not Found`.
 Тело ответа может содержать сообщение об ошибке, например:
 -invalid_id`
@@ -1103,12 +908,6 @@
 3. Проверить тело ответа.</t>
   </si>
   <si>
-    <t>Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-ID товара: `abc`</t>
-  </si>
-  <si>
     <t>Сервер не должен выполнять удаление, так как ID товара имеет некорректный формат.
 Сервер должен вернуть ошибку, например:
 `400 Bad Request` или: `404 Not Found`
@@ -1196,38 +995,6 @@
 3. Проверить тело ответа.
 4. Отправить GET-запрос: GET `{{baseurl}}/api/products/879902`
 5. Проверить, что карточка товара осталась доступна и не была изменена.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Авторизация:
-Login: skillboxadmin
-Password: iamfinallytester
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(НО В КОЛЛЕКЦИИ DELETE ЗАПРОСОВ ЭТИ ДАННЫЕ НЕ ВВЕДЕНЫ)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-ID товара: `879902`
-</t>
-    </r>
   </si>
   <si>
     <t>Сервер должен запретить удаление товара без авторизации.
@@ -1321,45 +1088,6 @@
 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Авторизация:
-Login</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">: skillboxadmin
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Password</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">: iamfinallytester
-</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">Карточка товара не создаётся.  
 Сервер возвращает ошибку обработки запроса, например `400 Bad Request`  или `415 Unsupported Media type` </t>
   </si>
@@ -1447,20 +1175,16 @@
 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Авторизация:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
+    <t xml:space="preserve">Карточка товара не создаётся.  
+Сервер возвращает ошибку обработки запроса, например `400 Bad Request` </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -1469,10 +1193,90 @@
       <rPr>
         <b/>
         <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">ДАННЫЕ ИЗМЕНЯЕМЫХ ПОЛЕЙ КАРТОЧКИ ТОВАРА ДО ИЗМЕНЕНИЙ:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">{
+    "name": "Поло для теста",
+    "description": "",
+    "price": "100",
+    "sale_price": "",
+    "images": [
+        {
+            "src": "http://intershop3.skillbox.ru/wp-content/uploads/2026/05/10564528-worried-fat-man-with-pink-shirt-isolated-on-white-background-19.jpg"
+        }
+    ]
+}
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">ДАННЫЕ ИЗМЕНЯЕМЫХ ПОЛЕЙ КАРТОЧКИ ТОВАРА ПОСЛЕ ИЗМЕНЕНИЙ:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>{
+  "name": "Поло мужское для теста",
+  "description": "Тестовое мужское поло для проверки редактирования карточки товара через PUT-запрос.",
+  "price": "85",
+  "sale_price": "85",
+  "images": [
+    {
+      "src": "</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://png.pngtree.com/png-clipart/20220815/ourmid/pngtree-mens-white-polo-shirt-for-clothing-model-mockup-and-passport-photo-png-image_6110906.png</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"
+    }
+  ]
+}
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Login:</t>
+      <t xml:space="preserve">
+Новое значение поля в PUT запросе
+</t>
     </r>
     <r>
       <rPr>
@@ -1480,7 +1284,19 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve"> skillboxadmin
+      <t>{
+  "id": 999999
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
     </r>
     <r>
@@ -1490,7 +1306,8 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Password:</t>
+      <t xml:space="preserve">Новое значение поля в PUT запросе
+</t>
     </r>
     <r>
       <rPr>
@@ -1498,7 +1315,23 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve"> iamfinallytester
+      <t>{
+  "price": hundred
+}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ID товара: `999999999`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ID товара получить из переменной {{productid}}
+Значение переменной `{{productid}}` взять из тестовой карточки товара.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
 </t>
     </r>
     <r>
@@ -1543,8 +1376,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Карточка товара не создаётся.  
-Сервер возвращает ошибку обработки запроса, например `400 Bad Request` </t>
+    <t xml:space="preserve">
+ID товара: `abc`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ID товара: `879902`
+</t>
   </si>
 </sst>
 </file>
@@ -1721,40 +1559,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1764,7 +1581,32 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2003,410 +1845,408 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="13" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:11" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" ht="261" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:11" ht="409.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="10" t="s">
+      <c r="C4" s="14"/>
+      <c r="D4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="9" t="s">
+    </row>
+    <row r="5" spans="1:11" ht="73.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" spans="1:11" ht="187.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-    </row>
-    <row r="6" spans="1:11" ht="187.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="B6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="14"/>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="10" t="s">
+      <c r="F6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="198" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="198" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="E7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="F7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="10" t="s">
+      <c r="G7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="198" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" s="10" t="s">
+      <c r="E8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="198" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="F8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="G8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="10" t="s">
+      <c r="H8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+    </row>
+    <row r="10" spans="1:11" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="D10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="E10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-    </row>
-    <row r="10" spans="1:11" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="F10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="G10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>17</v>
+      <c r="I10" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+    </row>
+    <row r="13" spans="1:11" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-    </row>
-    <row r="13" spans="1:11" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="F13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="G13" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="10" t="s">
+      <c r="I13" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="B14" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="C14" s="14"/>
+      <c r="D14" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="E14" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="F14" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="I13" s="9" t="s">
-        <v>17</v>
+      <c r="G14" s="4" t="s">
+        <v>78</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="H14" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="I14" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="158.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="9" t="s">
+      <c r="B15" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="C15" s="14"/>
+      <c r="D15" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="E15" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="F15" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="G15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>37</v>
+      <c r="I15" s="4" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+    <row r="16" spans="1:11" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+    </row>
+    <row r="17" spans="1:11" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+    </row>
+    <row r="18" spans="1:11" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="C18" s="7"/>
+      <c r="D18" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="E18" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="F18" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="G18" s="7"/>
+      <c r="H18" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="9" t="s">
-        <v>37</v>
+      <c r="I18" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-    </row>
-    <row r="17" spans="1:11" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="s">
+    <row r="19" spans="1:11" ht="369.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-    </row>
-    <row r="18" spans="1:11" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+      <c r="C19" s="7"/>
+      <c r="D19" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="E19" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="17" t="s">
+      <c r="F19" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="G19" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="H18" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="I18" s="16" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="409.2" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="G19" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="H19" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="I19" s="16" t="s">
-        <v>17</v>
+      <c r="I19" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -10135,11 +9975,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A17:I17"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="A1:A2"/>
@@ -10149,10 +9984,15 @@
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A17:I17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId2" display="Авторизация:_x000a_Login: skillboxadmin_x000a_Password: iamfinallytester_x000a__x000a_ДАННЫЕ ИЗМЕНЯЕМЫХ ПОЛЕЙ КАРТОЧКИ ТОВАРА ДО ИЗМЕНЕНИЙ:_x000a__x000a_{_x000a_    &quot;name&quot;: &quot;Поло для теста&quot;,_x000a_    &quot;description&quot;: &quot;&quot;,_x000a_    &quot;price&quot;: &quot;100&quot;,_x000a_    &quot;sale_price&quot;: &quot;&quot;,_x000a_    &quot;images&quot;: [_x000a_        {_x000a_            &quot;sr" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="H4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="E6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="E7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>

</xml_diff>